<commit_message>
MIDDLE - fixed xls-002 case
</commit_message>
<xml_diff>
--- a/tasks/excel/xls-002-sentiment1/solution/data/orders.xlsx
+++ b/tasks/excel/xls-002-sentiment1/solution/data/orders.xlsx
@@ -2,33 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -56,7 +51,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -421,10 +416,6 @@
   </sheetPr>
   <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="10.140625" bestFit="1" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -480,47 +471,47 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E2" t="n">
         <v>39</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Please confirm delivery date</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>All is good</t>
+          <t>Product works perfectly</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -532,12 +523,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -546,26 +537,26 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="E4" t="n">
         <v>39</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Tracking number not received</t>
+          <t>Will order again</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -579,31 +570,31 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="E5" t="n">
         <v>39</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Where is my invoice</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -612,14 +603,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>98</v>
+        <v>19</v>
       </c>
       <c r="E6" t="n">
         <v>39</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Where is my invoice</t>
+          <t>How to return the item</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -631,40 +622,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>117</v>
+        <v>26</v>
       </c>
       <c r="E7" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Item arrived broken</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -674,30 +665,30 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>136</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Would not recommend</t>
+          <t>Very satisfied</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -711,59 +702,59 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>155</v>
+        <v>44</v>
       </c>
       <c r="E9" t="n">
         <v>39</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Is warranty included</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-32</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>174</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>All is bad</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-35</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -773,18 +764,18 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>193</v>
+        <v>34</v>
       </c>
       <c r="E11" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Will order again</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -796,78 +787,78 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-38</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>212</v>
+        <v>18</v>
       </c>
       <c r="E12" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-41</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>231</v>
+        <v>16</v>
       </c>
       <c r="E13" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>Item arrived broken</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-44</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -876,14 +867,14 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
         <v>39</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Terrible support</t>
+          <t>All is bad</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -895,28 +886,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-47</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>269</v>
+        <v>44</v>
       </c>
       <c r="E15" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Would not recommend</t>
+          <t>Item arrived broken</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -928,61 +919,61 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-50</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>288</v>
+        <v>40</v>
       </c>
       <c r="E16" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>Tracking number not received</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-53</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>307</v>
+        <v>15</v>
       </c>
       <c r="E17" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Slow shipping</t>
+          <t>Terrible support</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -994,28 +985,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-56</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>326</v>
+        <v>31</v>
       </c>
       <c r="E18" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1027,94 +1018,94 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-59</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>345</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Would not recommend</t>
+          <t>Great service</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-62</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>364</v>
+        <v>39</v>
       </c>
       <c r="E20" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>All is good</t>
+          <t>All is bad</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-65</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>383</v>
+        <v>33</v>
       </c>
       <c r="E21" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Would not recommend</t>
+          <t>Too expensive for this quality</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1126,57 +1117,57 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-68</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>402</v>
+        <v>32</v>
       </c>
       <c r="E22" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>Slow shipping</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-71</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>421</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1192,61 +1183,61 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-74</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>440</v>
+        <v>15</v>
       </c>
       <c r="E24" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Do you have this in black</t>
+          <t>Will order again</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-77</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>459</v>
+        <v>36</v>
       </c>
       <c r="E25" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Slow shipping</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1258,12 +1249,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-80</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1272,76 +1263,76 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>478</v>
+        <v>30</v>
       </c>
       <c r="E26" t="n">
         <v>39</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Fast delivery, thanks</t>
+          <t>Please confirm delivery date</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-83</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>497</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>All is good</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-86</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>516</v>
+        <v>31</v>
       </c>
       <c r="E28" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1357,7 +1348,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-89</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1367,18 +1358,18 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>535</v>
+        <v>8</v>
       </c>
       <c r="E29" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Terrible support</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1390,73 +1381,73 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-92</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>554</v>
+        <v>30</v>
       </c>
       <c r="E30" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Is warranty included</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-95</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>573</v>
+        <v>39</v>
       </c>
       <c r="E31" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-98</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1466,47 +1457,47 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>592</v>
+        <v>48</v>
       </c>
       <c r="E32" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>How to return the item</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-101</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>611</v>
+        <v>36</v>
       </c>
       <c r="E33" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1522,7 +1513,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-104</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1532,68 +1523,68 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>630</v>
+        <v>23</v>
       </c>
       <c r="E34" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Too expensive for this quality</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-107</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>649</v>
+        <v>42</v>
       </c>
       <c r="E35" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Would not recommend</t>
+          <t>Great service</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-110</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1602,14 +1593,14 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>668</v>
+        <v>47</v>
       </c>
       <c r="E36" t="n">
         <v>39</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1621,61 +1612,61 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-113</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>687</v>
+        <v>42</v>
       </c>
       <c r="E37" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Please confirm delivery date</t>
+          <t>Very satisfied</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-116</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>706</v>
+        <v>19</v>
       </c>
       <c r="E38" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Item arrived broken</t>
+          <t>Slow shipping</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1687,73 +1678,73 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-119</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>725</v>
+        <v>25</v>
       </c>
       <c r="E39" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-122</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>744</v>
+        <v>22</v>
       </c>
       <c r="E40" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>All is good</t>
+          <t>Item arrived broken</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-125</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1763,18 +1754,18 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>763</v>
+        <v>24</v>
       </c>
       <c r="E41" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Great service</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1786,7 +1777,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-128</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1796,18 +1787,18 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>782</v>
+        <v>38</v>
       </c>
       <c r="E42" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Will order again</t>
+          <t>Very satisfied</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1819,12 +1810,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-131</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1833,14 +1824,14 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>801</v>
+        <v>14</v>
       </c>
       <c r="E43" t="n">
         <v>39</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1852,94 +1843,94 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-134</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>820</v>
+        <v>29</v>
       </c>
       <c r="E44" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>Please confirm delivery date</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-137</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>839</v>
+        <v>40</v>
       </c>
       <c r="E45" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Please confirm delivery date</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-140</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>858</v>
+        <v>12</v>
       </c>
       <c r="E46" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>All is bad</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1951,94 +1942,94 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-143</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>877</v>
+        <v>41</v>
       </c>
       <c r="E47" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Slow shipping</t>
+          <t>Is warranty included</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-146</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>896</v>
+        <v>19</v>
       </c>
       <c r="E48" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Slow shipping</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-149</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>915</v>
+        <v>30</v>
       </c>
       <c r="E49" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>Will order again</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2050,12 +2041,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-152</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2064,14 +2055,14 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>934</v>
+        <v>17</v>
       </c>
       <c r="E50" t="n">
         <v>39</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>Great service</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2083,61 +2074,61 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-155</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>953</v>
+        <v>4</v>
       </c>
       <c r="E51" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Terrible support</t>
+          <t>Great service</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-158</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>972</v>
+        <v>24</v>
       </c>
       <c r="E52" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Do you have this in black</t>
+          <t>Tracking number not received</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2149,12 +2140,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-161</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2163,80 +2154,80 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>991</v>
+        <v>27</v>
       </c>
       <c r="E53" t="n">
         <v>39</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Too expensive for this quality</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-164</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1010</v>
+        <v>43</v>
       </c>
       <c r="E54" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Do you have this in black</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-167</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1029</v>
+        <v>18</v>
       </c>
       <c r="E55" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2248,127 +2239,127 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-170</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1048</v>
+        <v>19</v>
       </c>
       <c r="E56" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Where is my invoice</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-173</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1067</v>
+        <v>33</v>
       </c>
       <c r="E57" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Where is my invoice</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-176</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1086</v>
+        <v>4</v>
       </c>
       <c r="E58" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Slow shipping</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-179</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1105</v>
+        <v>42</v>
       </c>
       <c r="E59" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Fast delivery, thanks</t>
+          <t>Product works perfectly</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2380,61 +2371,61 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-182</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1124</v>
+        <v>17</v>
       </c>
       <c r="E60" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Where is my invoice</t>
+          <t>Product works perfectly</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-185</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1143</v>
+        <v>14</v>
       </c>
       <c r="E61" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Too expensive for this quality</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2446,28 +2437,28 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-188</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1162</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Will order again</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2479,7 +2470,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-191</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2489,30 +2480,30 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1181</v>
+        <v>50</v>
       </c>
       <c r="E63" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Very satisfied</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-194</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2522,30 +2513,30 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1200</v>
+        <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Do you have this in black</t>
+          <t>Very satisfied</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-197</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2555,18 +2546,18 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1219</v>
+        <v>22</v>
       </c>
       <c r="E65" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Product works perfectly</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2578,28 +2569,28 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-200</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1238</v>
+        <v>19</v>
       </c>
       <c r="E66" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2611,12 +2602,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-203</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2625,14 +2616,14 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1257</v>
+        <v>11</v>
       </c>
       <c r="E67" t="n">
         <v>39</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2644,57 +2635,57 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-206</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1276</v>
+        <v>34</v>
       </c>
       <c r="E68" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Will order again</t>
+          <t>Is warranty included</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-209</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1295</v>
+        <v>41</v>
       </c>
       <c r="E69" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2710,78 +2701,78 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-212</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1314</v>
+        <v>42</v>
       </c>
       <c r="E70" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Tracking number not received</t>
+          <t>Item arrived broken</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-215</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1333</v>
+        <v>5</v>
       </c>
       <c r="E71" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Do you have this in black</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-218</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2790,26 +2781,26 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>1352</v>
+        <v>29</v>
       </c>
       <c r="E72" t="n">
         <v>39</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Fast delivery, thanks</t>
+          <t>Terrible support</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-221</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2819,35 +2810,35 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1371</v>
+        <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Tracking number not received</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-08-224</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2856,7 +2847,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1390</v>
+        <v>32</v>
       </c>
       <c r="E74" t="n">
         <v>39</v>
@@ -2875,12 +2866,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-08-227</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2889,80 +2880,80 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1409</v>
+        <v>17</v>
       </c>
       <c r="E75" t="n">
         <v>39</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Fast delivery, thanks</t>
+          <t>Too expensive for this quality</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-08-230</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1428</v>
+        <v>48</v>
       </c>
       <c r="E76" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-08-233</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1447</v>
+        <v>34</v>
       </c>
       <c r="E77" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2974,28 +2965,28 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-08-236</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1466</v>
+        <v>41</v>
       </c>
       <c r="E78" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>Fast delivery, thanks</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3007,12 +2998,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-08-239</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3021,64 +3012,64 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1485</v>
+        <v>2</v>
       </c>
       <c r="E79" t="n">
         <v>39</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Please confirm delivery date</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-08-242</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1504</v>
+        <v>36</v>
       </c>
       <c r="E80" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Will order again</t>
+          <t>Slow shipping</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-08-245</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3087,47 +3078,47 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1523</v>
+        <v>27</v>
       </c>
       <c r="E81" t="n">
         <v>39</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Where is my invoice</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-08-248</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1542</v>
+        <v>34</v>
       </c>
       <c r="E82" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Do you have this in black</t>
+          <t>How to return the item</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3139,12 +3130,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-08-251</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3153,14 +3144,14 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1561</v>
+        <v>44</v>
       </c>
       <c r="E83" t="n">
         <v>39</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>All is bad</t>
+          <t>Too expensive for this quality</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3172,45 +3163,45 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-08-254</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1580</v>
+        <v>45</v>
       </c>
       <c r="E84" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Is warranty included</t>
+          <t>Item arrived broken</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-08-257</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3219,7 +3210,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1599</v>
+        <v>45</v>
       </c>
       <c r="E85" t="n">
         <v>39</v>
@@ -3238,40 +3229,40 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-08-260</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>1618</v>
+        <v>38</v>
       </c>
       <c r="E86" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Great service</t>
+          <t>All is bad</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-08-263</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3285,31 +3276,31 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1637</v>
+        <v>28</v>
       </c>
       <c r="E87" t="n">
         <v>39</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Where is my invoice</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-08-266</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3318,14 +3309,14 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>1656</v>
+        <v>23</v>
       </c>
       <c r="E88" t="n">
         <v>39</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Item arrived broken</t>
+          <t>Slow shipping</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3337,12 +3328,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-08-269</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3351,14 +3342,14 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>1675</v>
+        <v>33</v>
       </c>
       <c r="E89" t="n">
         <v>39</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>All is bad</t>
+          <t>Would not recommend</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3370,7 +3361,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-08-272</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3380,30 +3371,30 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1694</v>
+        <v>35</v>
       </c>
       <c r="E90" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Fast delivery, thanks</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-08-275</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3413,35 +3404,35 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1713</v>
+        <v>18</v>
       </c>
       <c r="E91" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Fast delivery, thanks</t>
+          <t>Tracking number not received</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>neutral</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-08-278</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3450,7 +3441,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>1732</v>
+        <v>35</v>
       </c>
       <c r="E92" t="n">
         <v>39</v>
@@ -3469,28 +3460,28 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-08-281</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1751</v>
+        <v>34</v>
       </c>
       <c r="E93" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>All is bad</t>
+          <t>Terrible support</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -3502,61 +3493,61 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-08-284</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>south</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>1770</v>
+        <v>33</v>
       </c>
       <c r="E94" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Please confirm delivery date</t>
+          <t>All is good</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-08-287</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>gadget-d</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1789</v>
+        <v>6</v>
       </c>
       <c r="E95" t="n">
-        <v>39</v>
+        <v>4.2</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Will order again</t>
+          <t>Great service</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -3568,7 +3559,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-08-290</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3578,18 +3569,18 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>1808</v>
+        <v>8</v>
       </c>
       <c r="E96" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Slow shipping</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -3601,40 +3592,40 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-08-293</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>1827</v>
+        <v>14</v>
       </c>
       <c r="E97" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>All is bad</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-08-296</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3648,59 +3639,59 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>1846</v>
+        <v>12</v>
       </c>
       <c r="E98" t="n">
         <v>39</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Is warranty included</t>
+          <t>Excellent quality</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-08-299</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>east</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-b</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>1865</v>
+        <v>12</v>
       </c>
       <c r="E99" t="n">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Excellent quality</t>
+          <t>Very disappointed</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-08-302</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3714,52 +3705,52 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1884</v>
+        <v>11</v>
       </c>
       <c r="E100" t="n">
         <v>39</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Very disappointed</t>
+          <t>Will order again</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-08-305</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>gadget-c</t>
+          <t>widget-a</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>1903</v>
+        <v>3</v>
       </c>
       <c r="E101" t="n">
-        <v>39</v>
+        <v>9.5</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Item arrived broken</t>
+          <t>Very satisfied</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3788,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -3807,7 +3798,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -3817,7 +3808,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>